<commit_message>
chore(hyu-jacket): 영어 주문서에 SR(M) 추가 — 11명
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_영어필기체.xlsx
+++ b/vendor-order/TJ300_영어필기체.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -376,6 +376,12 @@
   </si>
   <si>
     <t xml:space="preserve">lofy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">omotinoyousei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR</t>
   </si>
 </sst>
 </file>
@@ -3578,7 +3584,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8">
@@ -4448,13 +4454,13 @@
         <v>8</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E83" s="2"/>
     </row>
@@ -4463,13 +4469,13 @@
         <v>9</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E84" s="2"/>
     </row>
@@ -4478,13 +4484,13 @@
         <v>10</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>103</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E85" s="2"/>
     </row>
@@ -4492,9 +4498,15 @@
       <c r="A86" s="2">
         <v>11</v>
       </c>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
+      <c r="B86" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="E86" s="2"/>
     </row>
     <row r="87" spans="1:5">

</xml_diff>

<commit_message>
chore(hyu-jacket): 영어 주문서에 WeiYitong(M) 추가 — 12명
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_영어필기체.xlsx
+++ b/vendor-order/TJ300_영어필기체.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="114">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -382,6 +382,12 @@
   </si>
   <si>
     <t xml:space="preserve">SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3433105578</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WeiYitong</t>
   </si>
 </sst>
 </file>
@@ -3584,7 +3590,7 @@
         <v>4</v>
       </c>
       <c r="D23" s="8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8">
@@ -4469,13 +4475,13 @@
         <v>9</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>96</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="E84" s="2"/>
     </row>
@@ -4484,13 +4490,13 @@
         <v>10</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E85" s="2"/>
     </row>
@@ -4499,13 +4505,13 @@
         <v>11</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>103</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E86" s="2"/>
     </row>
@@ -4513,9 +4519,15 @@
       <c r="A87" s="2">
         <v>12</v>
       </c>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
+      <c r="B87" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="E87" s="2"/>
     </row>
     <row r="88" spans="1:5">

</xml_diff>